<commit_message>
Selesai running dan analisis ulang hulu ke hilir.
</commit_message>
<xml_diff>
--- a/outputs/metrics/baseline_default_test_metrics.xlsx
+++ b/outputs/metrics/baseline_default_test_metrics.xlsx
@@ -610,40 +610,40 @@
         <v>0.5</v>
       </c>
       <c r="D4" t="n">
-        <v>0.7312703583061889</v>
+        <v>0.7214983713355049</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6788321167883211</v>
+        <v>0.6678832116788321</v>
       </c>
       <c r="F4" t="n">
-        <v>0.7072243346007605</v>
+        <v>0.6958174904942965</v>
       </c>
       <c r="G4" t="n">
-        <v>0.3211678832116788</v>
+        <v>0.3321167883211679</v>
       </c>
       <c r="H4" t="n">
-        <v>0.6927374301675978</v>
+        <v>0.6815642458100558</v>
       </c>
       <c r="I4" t="n">
-        <v>0.7492877492877493</v>
+        <v>0.7407407407407407</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5299145299145299</v>
+        <v>0.5169491525423728</v>
       </c>
       <c r="K4" t="n">
-        <v>0.7971087495802325</v>
+        <v>0.7962421327440339</v>
       </c>
       <c r="L4" t="n">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="M4" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="N4" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="O4" t="n">
-        <v>186</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>